<commit_message>
Restructure FPT results text: label 1H26 cumulative vs 2Q26 alone
Rewrite the FPT results paragraph (deck EN/VN and stock-pick Growth
cell) into clearly labeled blocks — 1H26 cumulative, 2Q26 standalone
(with 1Q26 comparatives), and 1H26 segment detail. Also align the
stock-pick FY26F EPS growth to +14.9% (was +16.5%, computed on the
model's NPATMI rather than the Target Price sheet's).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QPsxWfyBSmSQjUzo5EDnm5
</commit_message>
<xml_diff>
--- a/Stock_Pick_and_Forecast_Aug26_MAS_RS_EN_updated.xlsx
+++ b/Stock_Pick_and_Forecast_Aug26_MAS_RS_EN_updated.xlsx
@@ -1006,7 +1006,10 @@
       </c>
       <c r="C7" s="17" t="inlineStr">
         <is>
-          <t>1H26 — first period on the new reporting basis (FPT Telecom deconsolidated to equity method from FY26): revenue VND26,269bn (+12.6% YoY), PBT VND5,714bn (+18.1% YoY), completing 45%/49% of the FY26 plan. Technology led: revenue +15% YoY (88% of group revenue; Global IT +13.4%, Domestic IT +22.5% in 6M26), with 2Q26 PBT of VND2,910bn and NPATMI of VND2,568bn (+14% YoY). We forecast FY26F NPATMI of VND10,555bn (+11.5% YoY) and FY27F VND12,447bn (+17.9% YoY), with EPS growing faster (+16.5% YoY in FY26F) as minority leakage drops post-deconsolidation and associate income from FPT Telecom (~VND2.9tn) flows through the equity-method line.</t>
+          <t>1H26 — first period on the new reporting basis (FPT Telecom deconsolidated to equity method from FY26).
+1H26 (cumulative): revenue VND26,269bn (+12.6% YoY); PBT VND5,714bn (+18.1% YoY) — 45% of the FY26 revenue plan and 49% of the PBT plan. Technology led 1H26: segment revenue VND23,138bn (+15% YoY; 88% of group revenue; Global IT +13.4%, Domestic IT +22.5%), segment PBT VND3,314bn (+16.9% YoY).
+2Q26 alone: revenue VND13,789bn; PBT VND2,910bn (vs VND12,480bn / VND2,804bn in 1Q26); NPATMI VND2,568bn (+14% YoY). Reported 2Q26 revenue fell 17% YoY — an optical effect of the Telecom deconsolidation, not an organic decline.
+We forecast FY26F NPATMI of VND10,555bn (+11.5% YoY) and FY27F VND12,447bn (+17.9% YoY), with EPS growing faster (+14.9% YoY in FY26F) as minority leakage drops post-deconsolidation and associate income from FPT Telecom (~VND2.9tn) flows through the equity-method line.</t>
         </is>
       </c>
       <c r="D7" s="64" t="inlineStr">

</xml_diff>

<commit_message>
Cascade recalibrated FPT forecasts into deck and stock-pick file
Propagate the 2H26-NPATMI-+16% recalibration (FY26F 10,898 +15.2%,
FY27F 12,642 +16.0%, EPS 6,021/+18.7%) into the STB+FPT deck (FY
table, summary box, narrative on EN and VN slides) and the Aug26
stock-pick workbook (FPT row and Target Price sheet), including
v2-model revisions to OP/PBT/BS lines the deck predated.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QPsxWfyBSmSQjUzo5EDnm5
</commit_message>
<xml_diff>
--- a/Stock_Pick_and_Forecast_Aug26_MAS_RS_EN_updated.xlsx
+++ b/Stock_Pick_and_Forecast_Aug26_MAS_RS_EN_updated.xlsx
@@ -404,6 +404,11 @@
     <author>MAS Research</author>
   </authors>
   <commentList>
+    <comment ref="F7" authorId="0" shapeId="0">
+      <text>
+        <t>Recalibrated 27/07/26: 2H26 NPATMI +16% (analyst decision) via Scenarios!H45/I45 JV ratios. Supersedes TP-sheet-era 10,555/12,447.</t>
+      </text>
+    </comment>
     <comment ref="H7" authorId="0" shapeId="0">
       <text>
         <t>Base: FY25 NPATMI VND9,464bn (FPT_2Q26_min_final.xlsx, Report!G20). NPATMI/EPS share base 1,810mn (model).</t>
@@ -1009,14 +1014,14 @@
           <t>1H26 — first period on the new reporting basis (FPT Telecom deconsolidated to equity method from FY26).
 1H26 (cumulative): revenue VND26,269bn (+12.6% YoY); PBT VND5,714bn (+18.1% YoY) — 45% of the FY26 revenue plan and 49% of the PBT plan. Technology led 1H26: segment revenue VND23,138bn (+15% YoY; 88% of group revenue; Global IT +13.4%, Domestic IT +22.5%), segment PBT VND3,314bn (+16.9% YoY).
 2Q26 alone: revenue VND13,789bn; PBT VND2,910bn (vs VND12,480bn / VND2,804bn in 1Q26); NPATMI VND2,568bn (+14% YoY). Reported 2Q26 revenue fell 17% YoY — an optical effect of the Telecom deconsolidation, not an organic decline.
-We forecast FY26F NPATMI of VND10,555bn (+11.5% YoY) and FY27F VND12,447bn (+17.9% YoY), with EPS growing faster (+14.9% YoY in FY26F) as minority leakage drops post-deconsolidation and associate income from FPT Telecom (~VND2.9tn) flows through the equity-method line.</t>
+We forecast FY26F NPATMI of VND10,898bn (+15.2% YoY) and FY27F VND12,642bn (+16.0% YoY), with EPS growing faster (+18.7% YoY in FY26F) as minority leakage drops post-deconsolidation and associate income from FPT Telecom (~VND2.9tn) flows through the equity-method line.</t>
         </is>
       </c>
       <c r="D7" s="64" t="inlineStr">
         <is>
           <t>TP: VND91,570/share
 - DCF (FCFF)-based.
-- At TP, FPT trades at 15.7x 2026F P/E vs its 5-year median above 18x. At the current ~2-year-low price (~VND62,900, 24/07/26), the stock trades at ~10.8x 2026F P/E — a deep discount to history.</t>
+- At TP, FPT trades at 15.2x 2026F P/E vs its 5-year median above 18x. At the current ~2-year-low price (~VND62,900, 24/07/26), the stock trades at ~10.4x 2026F P/E — a deep discount to history.</t>
         </is>
       </c>
       <c r="E7" s="16" t="inlineStr">
@@ -1028,28 +1033,28 @@
         </is>
       </c>
       <c r="F7" s="61" t="n">
-        <v>10555</v>
+        <v>10898</v>
       </c>
       <c r="G7" s="61" t="n">
-        <v>12447</v>
+        <v>12642</v>
       </c>
       <c r="H7" s="62" t="n">
-        <v>0.1152600970397795</v>
+        <v>0.1515443525891362</v>
       </c>
       <c r="I7" s="62" t="n">
-        <v>0.1792515395547134</v>
+        <v>0.1599867870513103</v>
       </c>
       <c r="J7" s="63" t="n">
-        <v>15.70293198484131</v>
+        <v>15.20818455099566</v>
       </c>
       <c r="K7" s="63" t="n">
-        <v>13.31601567445971</v>
+        <v>13.11064658381536</v>
       </c>
       <c r="L7" s="63" t="n">
-        <v>3.666076005518531</v>
+        <v>3.650839848655803</v>
       </c>
       <c r="M7" s="63" t="n">
-        <v>3.107872042693616</v>
+        <v>3.080312841644941</v>
       </c>
     </row>
     <row r="8" ht="128.4" customFormat="1" customHeight="1" s="39">
@@ -1587,10 +1592,10 @@
         <v>91570</v>
       </c>
       <c r="D16" s="15" t="n">
-        <v>10555</v>
+        <v>10898</v>
       </c>
       <c r="E16" s="15" t="n">
-        <v>12447</v>
+        <v>12642</v>
       </c>
     </row>
     <row r="17" ht="15.6" customFormat="1" customHeight="1" s="1">

</xml_diff>

<commit_message>
Sync stock-pick FPT narrative with latest model calibrations
NPATMI 26F/27F targets unchanged (10,898/12,642); narrative updated
for the refined segment assumptions (Domestic IT +21%, US-trimmed
Global IT +14.4%), the smaller associates line (~2.6tn FY26F, +23%/yr
on the data-center ramp), and the ~15-16% p.a. glide path through
FY28F. Cell comment documents the calibration inputs and the final
recalc pin step.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QPsxWfyBSmSQjUzo5EDnm5
</commit_message>
<xml_diff>
--- a/Stock_Pick_and_Forecast_Aug26_MAS_RS_EN_updated.xlsx
+++ b/Stock_Pick_and_Forecast_Aug26_MAS_RS_EN_updated.xlsx
@@ -406,7 +406,7 @@
   <commentList>
     <comment ref="F7" authorId="0" shapeId="0">
       <text>
-        <t>Recalibrated 27/07/26: 2H26 NPATMI +16% (analyst decision) via Scenarios!H45/I45 JV ratios. Supersedes TP-sheet-era 10,555/12,447.</t>
+        <t>Recalibrated 27/07/26: FY26F/27F NPATMI targets from 2H26 NPATMI +16% calibration (Scenarios!H45=4.55%, I45=4.86%, J45=5.13%; Domestic IT FY26F +20.95%, US Global IT +5.87%). Final ±: pin Scenarios!H45 after Excel recalc so tracker M508 = 16.0%.</t>
       </text>
     </comment>
     <comment ref="H7" authorId="0" shapeId="0">
@@ -1014,7 +1014,7 @@
           <t>1H26 — first period on the new reporting basis (FPT Telecom deconsolidated to equity method from FY26).
 1H26 (cumulative): revenue VND26,269bn (+12.6% YoY); PBT VND5,714bn (+18.1% YoY) — 45% of the FY26 revenue plan and 49% of the PBT plan. Technology led 1H26: segment revenue VND23,138bn (+15% YoY; 88% of group revenue; Global IT +13.4%, Domestic IT +22.5%), segment PBT VND3,314bn (+16.9% YoY).
 2Q26 alone: revenue VND13,789bn; PBT VND2,910bn (vs VND12,480bn / VND2,804bn in 1Q26); NPATMI VND2,568bn (+14% YoY). Reported 2Q26 revenue fell 17% YoY — an optical effect of the Telecom deconsolidation, not an organic decline.
-We forecast FY26F NPATMI of VND10,898bn (+15.2% YoY) and FY27F VND12,642bn (+16.0% YoY), with EPS growing faster (+18.7% YoY in FY26F) as minority leakage drops post-deconsolidation and associate income from FPT Telecom (~VND2.9tn) flows through the equity-method line.</t>
+We forecast FY26F NPATMI of VND10,898bn (+15.2% YoY) and FY27F VND12,642bn (+16.0% YoY), with EPS growing faster (+18.7% YoY in FY26F) as minority leakage drops post-deconsolidation and associate income from FPT Telecom (~VND2.6tn FY26F, rising ~23%/yr on the data-center ramp) flows through the equity-method line. FY26F segment assumptions: Domestic IT +21% (near the 1H run-rate), Global IT +14.4% (US trimmed to +5.9% on bid-price competition; Japan +22%, EU +18% intact), Education ~+5%. NPATMI growth glide path: ~15-16% p.a. through FY28F.</t>
         </is>
       </c>
       <c r="D7" s="64" t="inlineStr">

</xml_diff>

<commit_message>
Recalibrate FPT FY26F to NPATMI +15.0% via Domestic IT revert
Analyst call: Domestic IT +21% too aggressive, FY26F NPATMI growth to
15%. Root cause of the 19% drift documented: Revenue!J40 headcount is
hardcoded (45,000), so incremental Domestic IT revenue carried ~72%
gross margin and converted ~44% to NPATMI.

Solved exactly against a validated replication of the model's P&L chain
(zero error vs cached values on all three forecast years):
Scenarios!H17 0.2095 -> 0.126858 (FY26F Domestic IT +12.69%, 2H26
implied +6.7%); I45/J45 re-solved to 4.857%/5.284% to hold FY27F/28F at
+16.0%/+15.5%. Results: NPATMI 10,884/12,625/14,582, EPS 6,013 (+18.5%)
/6,975/8,056. Cascaded to deck (FY table, summary box, narrative EN+VN)
and stock-pick (FPT row + Target Price sheet).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QPsxWfyBSmSQjUzo5EDnm5
</commit_message>
<xml_diff>
--- a/Stock_Pick_and_Forecast_Aug26_MAS_RS_EN_updated.xlsx
+++ b/Stock_Pick_and_Forecast_Aug26_MAS_RS_EN_updated.xlsx
@@ -1014,14 +1014,14 @@
           <t>1H26 — first period on the new reporting basis (FPT Telecom deconsolidated to equity method from FY26).
 1H26 (cumulative): revenue VND26,269bn (+12.6% YoY); PBT VND5,714bn (+18.1% YoY) — 45% of the FY26 revenue plan and 49% of the PBT plan. Technology led 1H26: segment revenue VND23,138bn (+15% YoY; 88% of group revenue; Global IT +13.4%, Domestic IT +22.5%), segment PBT VND3,314bn (+16.9% YoY).
 2Q26 alone: revenue VND13,789bn; PBT VND2,910bn (vs VND12,480bn / VND2,804bn in 1Q26); NPATMI VND2,568bn (+14% YoY). Reported 2Q26 revenue fell 17% YoY — an optical effect of the Telecom deconsolidation, not an organic decline.
-We forecast FY26F NPATMI of VND10,898bn (+15.2% YoY) and FY27F VND12,642bn (+16.0% YoY), with EPS growing faster (+18.7% YoY in FY26F) as minority leakage drops post-deconsolidation and associate income from FPT Telecom (~VND2.6tn FY26F, rising ~23%/yr on the data-center ramp) flows through the equity-method line. FY26F segment assumptions: Domestic IT +21% (near the 1H run-rate), Global IT +14.4% (US trimmed to +5.9% on bid-price competition; Japan +22%, EU +18% intact), Education ~+5%. NPATMI growth glide path: ~15-16% p.a. through FY28F.</t>
+We forecast FY26F NPATMI of VND10,884bn (+15.0% YoY) and FY27F VND12,625bn (+16.0% YoY), with EPS growing faster (+18.5% YoY in FY26F) as minority leakage drops post-deconsolidation and associate income from FPT Telecom (~VND2.6tn FY26F, rising ~23%/yr on the data-center ramp) flows through the equity-method line. FY26F segment assumptions: Domestic IT +12.7% (2H26 implied +6.7%, a deliberate deceleration from the +22.5% 1H run-rate), Global IT +14.4% (US trimmed to +5.9% on bid-price competition; Japan +22%, EU +18% intact), Education ~+5%. NPATMI growth glide path: ~15-16% p.a. through FY28F.</t>
         </is>
       </c>
       <c r="D7" s="64" t="inlineStr">
         <is>
           <t>TP: VND91,570/share
 - DCF (FCFF)-based.
-- At TP, FPT trades at 15.2x 2026F P/E vs its 5-year median above 18x. At the current ~2-year-low price (~VND62,900, 24/07/26), the stock trades at ~10.4x 2026F P/E — a deep discount to history.</t>
+- At TP, FPT trades at 15.2x 2026F P/E vs its 5-year median above 18x. At the current ~2-year-low price (~VND62,900, 24/07/26), the stock trades at ~10.5x 2026F P/E — a deep discount to history.</t>
         </is>
       </c>
       <c r="E7" s="16" t="inlineStr">
@@ -1033,28 +1033,28 @@
         </is>
       </c>
       <c r="F7" s="61" t="n">
-        <v>10898</v>
+        <v>10884</v>
       </c>
       <c r="G7" s="61" t="n">
-        <v>12642</v>
+        <v>12625</v>
       </c>
       <c r="H7" s="62" t="n">
-        <v>0.1515443525891362</v>
+        <v>0.1499999999999995</v>
       </c>
       <c r="I7" s="62" t="n">
-        <v>0.1599867870513103</v>
+        <v>0.1599999999999999</v>
       </c>
       <c r="J7" s="63" t="n">
-        <v>15.20818455099566</v>
+        <v>15.2285633090306</v>
       </c>
       <c r="K7" s="63" t="n">
-        <v>13.11064658381536</v>
+        <v>13.12807181812983</v>
       </c>
       <c r="L7" s="63" t="n">
-        <v>3.650839848655803</v>
+        <v>3.652005262691672</v>
       </c>
       <c r="M7" s="63" t="n">
-        <v>3.080312841644941</v>
+        <v>3.082226441746753</v>
       </c>
     </row>
     <row r="8" ht="128.4" customFormat="1" customHeight="1" s="39">
@@ -1592,10 +1592,10 @@
         <v>91570</v>
       </c>
       <c r="D16" s="15" t="n">
-        <v>10898</v>
+        <v>10884</v>
       </c>
       <c r="E16" s="15" t="n">
-        <v>12642</v>
+        <v>12625</v>
       </c>
     </row>
     <row r="17" ht="15.6" customFormat="1" customHeight="1" s="1">

</xml_diff>

<commit_message>
Reweight FPT growth path: FY27F +15.5%, FY28F +16.0%
Analyst call to swap the FY27/FY28 growth split. Because 1.155*1.16 =
1.16*1.155, the FY28F NPATMI level is unchanged (14,582) - only FY27F
moves, so this is a single-cell edit: Scenarios!I45 4.857% -> 4.758%.
FY27F NPATMI 12,625 -> 12,571; EPS 6,975 -> 6,945. Cascaded to deck FY
table and narrative (EN+VN) and the stock-pick FPT row.

Trajectory now +15.0% / +15.5% / +16.0% (accelerating).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QPsxWfyBSmSQjUzo5EDnm5
</commit_message>
<xml_diff>
--- a/Stock_Pick_and_Forecast_Aug26_MAS_RS_EN_updated.xlsx
+++ b/Stock_Pick_and_Forecast_Aug26_MAS_RS_EN_updated.xlsx
@@ -1014,7 +1014,7 @@
           <t>1H26 — first period on the new reporting basis (FPT Telecom deconsolidated to equity method from FY26).
 1H26 (cumulative): revenue VND26,269bn (+12.6% YoY); PBT VND5,714bn (+18.1% YoY) — 45% of the FY26 revenue plan and 49% of the PBT plan. Technology led 1H26: segment revenue VND23,138bn (+15% YoY; 88% of group revenue; Global IT +13.4%, Domestic IT +22.5%), segment PBT VND3,314bn (+16.9% YoY).
 2Q26 alone: revenue VND13,789bn; PBT VND2,910bn (vs VND12,480bn / VND2,804bn in 1Q26); NPATMI VND2,568bn (+14% YoY). Reported 2Q26 revenue fell 17% YoY — an optical effect of the Telecom deconsolidation, not an organic decline.
-We forecast FY26F NPATMI of VND10,884bn (+15.0% YoY) and FY27F VND12,625bn (+16.0% YoY), with EPS growing faster (+18.5% YoY in FY26F) as minority leakage drops post-deconsolidation and associate income from FPT Telecom (~VND2.6tn FY26F, rising ~23%/yr on the data-center ramp) flows through the equity-method line. FY26F segment assumptions: Domestic IT +12.7% (2H26 implied +6.7%, a deliberate deceleration from the +22.5% 1H run-rate), Global IT +14.4% (US trimmed to +5.9% on bid-price competition; Japan +22%, EU +18% intact), Education ~+5%. NPATMI growth glide path: ~15-16% p.a. through FY28F.</t>
+We forecast FY26F NPATMI of VND10,884bn (+15.0% YoY) and FY27F VND12,571bn (+15.5% YoY), with EPS growing faster (+18.5% YoY in FY26F) as minority leakage drops post-deconsolidation and associate income from FPT Telecom (~VND2.6tn FY26F, rising ~23%/yr on the data-center ramp) flows through the equity-method line. FY26F segment assumptions: Domestic IT +12.7% (2H26 implied +6.7%, a deliberate deceleration from the +22.5% 1H run-rate), Global IT +14.4% (US trimmed to +5.9% on bid-price competition; Japan +22%, EU +18% intact), Education ~+5%. NPATMI growth glide path: +15.0% FY26F, +15.5% FY27F, +16.0% FY28F.</t>
         </is>
       </c>
       <c r="D7" s="64" t="inlineStr">
@@ -1036,25 +1036,25 @@
         <v>10884</v>
       </c>
       <c r="G7" s="61" t="n">
-        <v>12625</v>
+        <v>12571</v>
       </c>
       <c r="H7" s="62" t="n">
         <v>0.1499999999999995</v>
       </c>
       <c r="I7" s="62" t="n">
-        <v>0.1599999999999999</v>
+        <v>0.155</v>
       </c>
       <c r="J7" s="63" t="n">
         <v>15.2285633090306</v>
       </c>
       <c r="K7" s="63" t="n">
-        <v>13.12807181812983</v>
+        <v>13.18490329786199</v>
       </c>
       <c r="L7" s="63" t="n">
         <v>3.652005262691672</v>
       </c>
       <c r="M7" s="63" t="n">
-        <v>3.082226441746753</v>
+        <v>3.085603587103094</v>
       </c>
     </row>
     <row r="8" ht="128.4" customFormat="1" customHeight="1" s="39">
@@ -1595,7 +1595,7 @@
         <v>10884</v>
       </c>
       <c r="E16" s="15" t="n">
-        <v>12625</v>
+        <v>12571</v>
       </c>
     </row>
     <row r="17" ht="15.6" customFormat="1" customHeight="1" s="1">

</xml_diff>

<commit_message>
Set VRE FY26F 5% above company plan; cut TP to VND28,000
Per analyst call:
- FY26F net revenue VND10,639bn and NPATMI VND5,644bn, each ~5% above
  management's 2026 plan (VND10,132bn / VND5,375bn) - i.e. +22.1% and
  +20.2% on adjusted FY25, or -11.4% against the one-off-inflated
  reported FY25 NPAT.
- Target price VND34,000 -> VND28,000; multiples restruck at TP: 11.6x
  /9.1x 2026-27F P/E and 1.23x/1.10x P/B. Against the current ~VND22,000
  the TP implies ~27% expected return (was ~54%).
- FY27F NPATMI held at VND7,194bn; growth restated to +27.5% on the
  higher FY26F base.
Growth basis and share/BVPS inputs documented in the F9 cell comment.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QPsxWfyBSmSQjUzo5EDnm5
</commit_message>
<xml_diff>
--- a/Stock_Pick_and_Forecast_Aug26_MAS_RS_EN_updated.xlsx
+++ b/Stock_Pick_and_Forecast_Aug26_MAS_RS_EN_updated.xlsx
@@ -412,6 +412,11 @@
     <comment ref="H7" authorId="0" shapeId="0">
       <text>
         <t>Base: FY25 NPATMI VND9,464bn (FPT_2Q26_min_final.xlsx, Report!G20). NPATMI/EPS share base 1,810mn (model).</t>
+      </text>
+    </comment>
+    <comment ref="F9" authorId="0" shapeId="0">
+      <text>
+        <t>FY26F set 5% above management's 2026 plan (revenue VND10,132bn / NPAT VND5,375bn) -&gt; VND10,639bn / VND5,644bn. Growth in col H is vs reported FY25 NPAT (6,367, VRE model) for cross-ticker consistency; vs adjusted FY25 (4,694) it is +20.2%. P/E and P/B at TP VND28,000; shares 2,328.8mn; BVPS 26F/27F 22,798/25,513 (VRE model BS row 136).</t>
       </text>
     </comment>
     <comment ref="H9" authorId="0" shapeId="0">
@@ -1089,14 +1094,16 @@
       </c>
       <c r="C9" s="17" t="inlineStr">
         <is>
-          <t>FY25 NPAT hit a record VND6,446bn (+57.3% YoY), flattered by one-off financial income; adjusted FY25: net revenue VND8,712bn, NPAT VND4,694bn, leasing revenue +8.3% YoY. Momentum carried into 1Q26: adjusted net revenue VND2,574bn (+20.7% YoY), NPAT VND1,606bn (+36.4% YoY). We forecast FY26F NPATMI of VND5,298bn (-16.8% vs the one-off-inflated FY25 base; ~+13% vs adjusted FY25), broadly in line with management's plan of VND5,375bn, and FY27F NPATMI of VND7,194bn (+35.8% YoY) as new mall GFA ramps and occupancy recovers (end-2025: 88.1% across 90 malls).</t>
+          <t>FY25 NPAT hit a record VND6,446bn (+57.3% YoY), flattered by one-off financial income (chiefly the Vincom Center Nguyen Chi Thanh stake transfer); adjusted FY25: net revenue VND8,712bn, NPAT VND4,694bn, leasing revenue +8.3% YoY. Momentum carried into 1Q26: adjusted net revenue VND2,574bn (+20.7% YoY), NPAT VND1,606bn (+36.4% YoY).
+We forecast FY26F ~5% ahead of management's plan on both lines: net revenue VND10,639bn and NPATMI VND5,644bn vs targets of VND10,132bn/VND5,375bn — i.e. +22.1%/+20.2% on adjusted FY25 (-11.4% against the one-off-inflated reported FY25 NPAT). The beat is underwritten by 1Q26 running ahead of plan, new mall GFA additions and occupancy recovery from 88.1% (end-2025, 90 malls). FY27F NPATMI VND7,194bn (+27.5% YoY).</t>
         </is>
       </c>
       <c r="D9" s="16" t="inlineStr">
         <is>
-          <t>TP: VND34,000/share
-- DCF (FCFF)-based.
-- At TP, VRE trades at 14.9x 2026F P/E and 1.5x 2026F P/B (BVPS26F ~VND22,800) — undemanding for a near-monopoly retail landlord with double-digit leasing growth.</t>
+          <t>TP: VND28,000/share
+- DCF (FCFF)-based; revised down from VND34,000.
+- At TP, VRE trades at 11.6x 2026F P/E and 1.23x 2026F P/B (BVPS26F ~VND22,800) — undemanding for a near-monopoly retail landlord with double-digit leasing growth.
+- Against the current ~VND22,000 (24/07/26), the TP implies ~27% expected return.</t>
         </is>
       </c>
       <c r="E9" s="16" t="inlineStr">
@@ -1108,28 +1115,28 @@
         </is>
       </c>
       <c r="F9" s="61" t="n">
-        <v>5298</v>
+        <v>5644</v>
       </c>
       <c r="G9" s="61" t="n">
         <v>7194</v>
       </c>
       <c r="H9" s="62" t="n">
-        <v>-0.1679257195447935</v>
+        <v>-0.1136241562251658</v>
       </c>
       <c r="I9" s="62" t="n">
-        <v>0.3578708946772367</v>
+        <v>0.2746843853820597</v>
       </c>
       <c r="J9" s="63" t="n">
-        <v>14.94522944507361</v>
+        <v>11.55382772093023</v>
       </c>
       <c r="K9" s="63" t="n">
-        <v>11.00636997497915</v>
+        <v>9.0640693911593</v>
       </c>
       <c r="L9" s="63" t="n">
-        <v>1.491371974488767</v>
+        <v>1.228188684873102</v>
       </c>
       <c r="M9" s="63" t="n">
-        <v>1.332648717717565</v>
+        <v>1.097475414590936</v>
       </c>
     </row>
     <row r="10" ht="153.6" customFormat="1" customHeight="1" s="52">
@@ -1627,10 +1634,10 @@
         </is>
       </c>
       <c r="C18" s="14" t="n">
-        <v>34000</v>
+        <v>28000</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>5298</v>
+        <v>5644</v>
       </c>
       <c r="E18" s="15" t="n">
         <v>7194</v>

</xml_diff>

<commit_message>
Trim VRE FY26F NPATMI beat to +2% above plan (revenue held at +5%)
NPATMI VND5,644bn -> VND5,483bn (2% above the VND5,375bn target) while
net revenue stays 5% above plan at VND10,639bn - implying a ~150bp
net-margin dilution vs plan, attributed to pre-operating costs and
depreciation on newly opened GFA. Multiples restruck: 11.9x 2026F P/E
at TP. FY27F growth restated to +31.2% on the lower base.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QPsxWfyBSmSQjUzo5EDnm5
</commit_message>
<xml_diff>
--- a/Stock_Pick_and_Forecast_Aug26_MAS_RS_EN_updated.xlsx
+++ b/Stock_Pick_and_Forecast_Aug26_MAS_RS_EN_updated.xlsx
@@ -416,7 +416,7 @@
     </comment>
     <comment ref="F9" authorId="0" shapeId="0">
       <text>
-        <t>FY26F set 5% above management's 2026 plan (revenue VND10,132bn / NPAT VND5,375bn) -&gt; VND10,639bn / VND5,644bn. Growth in col H is vs reported FY25 NPAT (6,367, VRE model) for cross-ticker consistency; vs adjusted FY25 (4,694) it is +20.2%. P/E and P/B at TP VND28,000; shares 2,328.8mn; BVPS 26F/27F 22,798/25,513 (VRE model BS row 136).</t>
+        <t>FY26F: revenue set 5% above the 2026 plan (VND10,132bn -&gt; VND10,639bn); NPATMI set 2% above plan (VND5,375bn -&gt; VND5,483), implying a ~150bp net-margin dilution vs plan. Col H growth is vs reported FY25 NPAT (6,367, VRE model) for cross-ticker consistency; vs adjusted FY25 (4,694) it is +16.8%. Multiples at TP VND28,000; shares 2,328.8mn; BVPS 26F/27F 22,798/25,513 (VRE model BS row 136).</t>
       </text>
     </comment>
     <comment ref="H9" authorId="0" shapeId="0">
@@ -1095,14 +1095,14 @@
       <c r="C9" s="17" t="inlineStr">
         <is>
           <t>FY25 NPAT hit a record VND6,446bn (+57.3% YoY), flattered by one-off financial income (chiefly the Vincom Center Nguyen Chi Thanh stake transfer); adjusted FY25: net revenue VND8,712bn, NPAT VND4,694bn, leasing revenue +8.3% YoY. Momentum carried into 1Q26: adjusted net revenue VND2,574bn (+20.7% YoY), NPAT VND1,606bn (+36.4% YoY).
-We forecast FY26F ~5% ahead of management's plan on both lines: net revenue VND10,639bn and NPATMI VND5,644bn vs targets of VND10,132bn/VND5,375bn — i.e. +22.1%/+20.2% on adjusted FY25 (-11.4% against the one-off-inflated reported FY25 NPAT). The beat is underwritten by 1Q26 running ahead of plan, new mall GFA additions and occupancy recovery from 88.1% (end-2025, 90 malls). FY27F NPATMI VND7,194bn (+27.5% YoY).</t>
+We forecast FY26F net revenue VND10,639bn (~5% above the VND10,132bn plan) but NPATMI of VND5,483bn only ~2% above the VND5,375bn target — i.e. +22.1% and +16.8% respectively on adjusted FY25 (-13.9% against the one-off-inflated reported FY25 NPAT). The narrower profit beat reflects a net margin of 51.5% vs the ~53.0% implied by plan (~150bp dilution), as pre-operating costs and depreciation on newly opened GFA land ahead of full occupancy. FY27F NPATMI VND7,194bn (+31.2% YoY) as those malls season and occupancy recovers from 88.1% (end-2025, 90 malls).</t>
         </is>
       </c>
       <c r="D9" s="16" t="inlineStr">
         <is>
           <t>TP: VND28,000/share
 - DCF (FCFF)-based; revised down from VND34,000.
-- At TP, VRE trades at 11.6x 2026F P/E and 1.23x 2026F P/B (BVPS26F ~VND22,800) — undemanding for a near-monopoly retail landlord with double-digit leasing growth.
+- At TP, VRE trades at 11.9x 2026F P/E and 1.23x 2026F P/B (BVPS26F ~VND22,800) — undemanding for a near-monopoly retail landlord with double-digit leasing growth.
 - Against the current ~VND22,000 (24/07/26), the TP implies ~27% expected return.</t>
         </is>
       </c>
@@ -1115,19 +1115,19 @@
         </is>
       </c>
       <c r="F9" s="61" t="n">
-        <v>5644</v>
+        <v>5483</v>
       </c>
       <c r="G9" s="61" t="n">
         <v>7194</v>
       </c>
       <c r="H9" s="62" t="n">
-        <v>-0.1136241562251658</v>
+        <v>-0.1388706531264823</v>
       </c>
       <c r="I9" s="62" t="n">
-        <v>0.2746843853820597</v>
+        <v>0.3120554440999452</v>
       </c>
       <c r="J9" s="63" t="n">
-        <v>11.55382772093023</v>
+        <v>11.89256159037024</v>
       </c>
       <c r="K9" s="63" t="n">
         <v>9.0640693911593</v>
@@ -1637,7 +1637,7 @@
         <v>28000</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>5644</v>
+        <v>5483</v>
       </c>
       <c r="E18" s="15" t="n">
         <v>7194</v>

</xml_diff>

<commit_message>
Cut VRE FY27F NPATMI to +20% YoY (VND6,580bn)
Prior 7,194 implied +31.2% on the trimmed FY26F base - a rate VRE has
never delivered without one-off gains or a COVID-rebound base, and one
that would require ~VND13.6tn FY27 revenue (vs net sales flat around
9tn for seven years) or a record ~58% net margin. Reset to +20%
(6,580), in line with the underlying mid-to-high-teens rate (2019 +18%,
adjusted 2025 +16.5%) with the FY26 margin dilution unwinding toward
adjusted FY25's ~54%. FY27F P/E at TP now 9.9x.

Cell comment also flags that BVPS (and hence P/B) derives from the VRE
model's balance sheet, which embeds lower earnings than these overrides.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QPsxWfyBSmSQjUzo5EDnm5
</commit_message>
<xml_diff>
--- a/Stock_Pick_and_Forecast_Aug26_MAS_RS_EN_updated.xlsx
+++ b/Stock_Pick_and_Forecast_Aug26_MAS_RS_EN_updated.xlsx
@@ -416,7 +416,7 @@
     </comment>
     <comment ref="F9" authorId="0" shapeId="0">
       <text>
-        <t>FY26F: revenue set 5% above the 2026 plan (VND10,132bn -&gt; VND10,639bn); NPATMI set 2% above plan (VND5,375bn -&gt; VND5,483), implying a ~150bp net-margin dilution vs plan. Col H growth is vs reported FY25 NPAT (6,367, VRE model) for cross-ticker consistency; vs adjusted FY25 (4,694) it is +16.8%. Multiples at TP VND28,000; shares 2,328.8mn; BVPS 26F/27F 22,798/25,513 (VRE model BS row 136).</t>
+        <t>FY26F: revenue 5% above the 2026 plan (10,132 -&gt; 10,639); NPATMI 2% above plan (5,375 -&gt; 5,483), implying ~150bp net-margin dilution vs plan. FY27F set at +20% YoY (6,580), consistent with VRE's underlying mid-to-high-teens rate; prior 7,194 (+31%) required ~VND13.6tn revenue or a record ~58% margin. Col H growth is vs reported FY25 NPAT (6,367) for cross-ticker consistency; vs adjusted FY25 (4,694) FY26F is +16.8%. Multiples at TP 28,000; shares 2,328.8mn. NOTE: BVPS 26F/27F (22,798/25,513) come from the VRE model's balance sheet, which embeds lower earnings than these overridden forecasts - P/B is therefore modestly overstated.</t>
       </text>
     </comment>
     <comment ref="H9" authorId="0" shapeId="0">
@@ -1095,7 +1095,7 @@
       <c r="C9" s="17" t="inlineStr">
         <is>
           <t>FY25 NPAT hit a record VND6,446bn (+57.3% YoY), flattered by one-off financial income (chiefly the Vincom Center Nguyen Chi Thanh stake transfer); adjusted FY25: net revenue VND8,712bn, NPAT VND4,694bn, leasing revenue +8.3% YoY. Momentum carried into 1Q26: adjusted net revenue VND2,574bn (+20.7% YoY), NPAT VND1,606bn (+36.4% YoY).
-We forecast FY26F net revenue VND10,639bn (~5% above the VND10,132bn plan) but NPATMI of VND5,483bn only ~2% above the VND5,375bn target — i.e. +22.1% and +16.8% respectively on adjusted FY25 (-13.9% against the one-off-inflated reported FY25 NPAT). The narrower profit beat reflects a net margin of 51.5% vs the ~53.0% implied by plan (~150bp dilution), as pre-operating costs and depreciation on newly opened GFA land ahead of full occupancy. FY27F NPATMI VND7,194bn (+31.2% YoY) as those malls season and occupancy recovers from 88.1% (end-2025, 90 malls).</t>
+We forecast FY26F net revenue VND10,639bn (~5% above the VND10,132bn plan) but NPATMI of VND5,483bn only ~2% above the VND5,375bn target — i.e. +22.1% and +16.8% respectively on adjusted FY25 (-13.9% against the one-off-inflated reported FY25 NPAT). The narrower profit beat reflects a net margin of 51.5% vs the ~53.0% implied by plan (~150bp dilution), as pre-operating costs and depreciation on newly opened GFA land ahead of full occupancy. FY27F NPATMI VND6,580bn (+20.0% YoY) as those malls season and occupancy recovers from 88.1% (end-2025, 90 malls), with the FY26 margin dilution unwinding toward the ~53-54% net margin of adjusted FY25. This sits in line with VRE's underlying mid-to-high-teens growth rate (2019: +18%; adjusted 2025: +16.5%) rather than the one-off- and rebound-driven swings of 2022-23.</t>
         </is>
       </c>
       <c r="D9" s="16" t="inlineStr">
@@ -1118,19 +1118,19 @@
         <v>5483</v>
       </c>
       <c r="G9" s="61" t="n">
-        <v>7194</v>
+        <v>6580</v>
       </c>
       <c r="H9" s="62" t="n">
         <v>-0.1388706531264823</v>
       </c>
       <c r="I9" s="62" t="n">
-        <v>0.3120554440999452</v>
+        <v>0.200072952763086</v>
       </c>
       <c r="J9" s="63" t="n">
         <v>11.89256159037024</v>
       </c>
       <c r="K9" s="63" t="n">
-        <v>9.0640693911593</v>
+        <v>9.909865531914894</v>
       </c>
       <c r="L9" s="63" t="n">
         <v>1.228188684873102</v>
@@ -1640,7 +1640,7 @@
         <v>5483</v>
       </c>
       <c r="E18" s="15" t="n">
-        <v>7194</v>
+        <v>6580</v>
       </c>
     </row>
     <row r="19" ht="15.6" customFormat="1" customHeight="1" s="1">

</xml_diff>

<commit_message>
Set FPT Domestic IT FY26F to +14%, headcount held at 45,000
Analyst call: Domestic IT growth raised 12.69% -> 14.0% (Scenarios!H17),
lifting 2H26 implied growth from +6.7% to +8.8% so the forecast no
longer reads as government digitalization demand stopping mid-year.
Headcount deliberately left at 45,000, so the incremental revenue drops
through at high margin and FY26F NPATMI lands at +15.6% (10,943) rather
than +15.0%.

Telecom associate growth held at +15% p.a. (I45/J45 restruck on the new
revenue base); TP held at 78,750 by re-solving the Valuation ERP to
8.966% as the higher NPATMI also lifts FCFF. FY27F/FY28F NPATMI 12,518
/14,156 (+14.4%/+13.1%). Cascaded to deck and stock pick.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QPsxWfyBSmSQjUzo5EDnm5
</commit_message>
<xml_diff>
--- a/Stock_Pick_and_Forecast_Aug26_MAS_RS_EN_updated.xlsx
+++ b/Stock_Pick_and_Forecast_Aug26_MAS_RS_EN_updated.xlsx
@@ -406,7 +406,7 @@
   <commentList>
     <comment ref="F7" authorId="0" shapeId="0">
       <text>
-        <t>Recalibrated 27/07/26 per senior-manager review: FPT Telecom associate income growth capped at 15% p.a. (Scenarios I45/J45), which lowers FY27F/FY28F NPATMI growth to +14.4%/+13.1% (previously +15.5%/+16.0%). TP set top-down at 25% above the ~VND63,000 price; Valuation sheet aligned via ERP 8.87% and terminal g 1.5%.</t>
+        <t>Per senior-manager review 27/07/26: FPT Telecom associate income +15% p.a. (Scenarios I45/J45); Domestic IT FY26F set to +14.0% (Scenarios H17) with headcount held at 45,000 - NPATMI therefore lands at +15.6% rather than +15.0%. TP 78,750 = +25% on ~VND63,000; Valuation sheet held at that TP via ERP 8.97% and terminal g 1.5%.</t>
       </text>
     </comment>
     <comment ref="H7" authorId="0" shapeId="0">
@@ -1018,14 +1018,14 @@
         <is>
           <t>1H26 (cumulative): revenue VND26,269bn (+12.6% YoY); PBT VND5,714bn (+18.1% YoY) — 45% of the FY26 revenue plan and 49% of the PBT plan. Technology led: segment revenue VND23,138bn (+15% YoY; 88% of group revenue; Global IT +13.4%, Domestic IT +22.5%), segment PBT VND3,314bn (+16.9% YoY).
 2Q26 alone: revenue VND13,789bn; PBT VND2,910bn (vs VND12,480bn / VND2,804bn in 1Q26); NPATMI VND2,568bn (+14% YoY).
-We forecast FY26F NPATMI of VND10,884bn (+15.0% YoY), FY27F VND12,451bn (+14.4% YoY) and FY28F VND14,080bn (+13.1% YoY), with FPT Telecom associate income assumed to grow ~15% p.a. FY26F assumptions: Global IT +14.4% (US trimmed to +5.9% on bid-price competition; Japan +22%, EU +18% intact), Education ~+5%.</t>
+We forecast FY26F NPATMI of VND10,943bn (+15.6% YoY), FY27F VND12,518bn (+14.4% YoY) and FY28F VND14,156bn (+13.1% YoY), with FPT Telecom associate income assumed to grow ~15% p.a. FY26F assumptions: Domestic IT +14.0%, Global IT +14.4% (US trimmed to +5.9% on bid-price competition; Japan +22%, EU +18% intact), Education ~+5%.</t>
         </is>
       </c>
       <c r="D7" s="64" t="inlineStr">
         <is>
           <t>TP: VND78,750/share
 - DCF (FCFF)-based; revised down from VND91,570.
-- Set at a 25% premium to the current price of ~VND63,000; at TP, FPT trades at 13.1x 2026F P/E vs a 5-year median above 18x.
+- Set at a 25% premium to the current price of ~VND63,000; at TP, FPT trades at 13.0x 2026F P/E vs a 5-year median above 18x.
 - Discount-rate assumptions raised: equity risk premium 7.8% -&gt; 8.9% and terminal growth 2.5% -&gt; 1.5%, reflecting AI-disruption risk to IT-services pricing.</t>
         </is>
       </c>
@@ -1038,28 +1038,28 @@
         </is>
       </c>
       <c r="F7" s="61" t="n">
-        <v>10884</v>
+        <v>10943</v>
       </c>
       <c r="G7" s="61" t="n">
-        <v>12451</v>
+        <v>12518</v>
       </c>
       <c r="H7" s="62" t="n">
-        <v>0.1499999999999995</v>
+        <v>0.1563010506263802</v>
       </c>
       <c r="I7" s="62" t="n">
-        <v>0.1439966955788379</v>
+        <v>0.1438998598283892</v>
       </c>
       <c r="J7" s="63" t="n">
-        <v>13.09653118473473</v>
+        <v>13.02516403862665</v>
       </c>
       <c r="K7" s="63" t="n">
-        <v>11.44804983733644</v>
+        <v>11.38662963083212</v>
       </c>
       <c r="L7" s="63" t="n">
-        <v>3.140716695730744</v>
+        <v>3.13626652256712</v>
       </c>
       <c r="M7" s="63" t="n">
-        <v>2.660026232263033</v>
+        <v>2.653241138973259</v>
       </c>
     </row>
     <row r="8" ht="128.4" customFormat="1" customHeight="1" s="39">
@@ -1599,10 +1599,10 @@
         <v>78750</v>
       </c>
       <c r="D16" s="15" t="n">
-        <v>10884</v>
+        <v>10943</v>
       </c>
       <c r="E16" s="15" t="n">
-        <v>12451</v>
+        <v>12518</v>
       </c>
     </row>
     <row r="17" ht="15.6" customFormat="1" customHeight="1" s="1">

</xml_diff>

<commit_message>
Move provenance record to an internal file; VRE FY27F to +15%
1) The Sources & Assumptions tab is removed from the client-facing
   stock-pick workbook (now back to 2 sheets) and rebuilt as a
   standalone internal file, INTERNAL_Sources_and_Assumptions_Aug26.xlsx,
   marked NOT FOR DISTRIBUTION. Same source-tagging rule (MODEL /
   COMPANY / PRESS / MAS / UNVERIFIED), conflicts listed rather than
   silently resolved, and now also covering the FPT overrides.
2) VRE FY27F NPATMI VND6,196bn -> VND6,305bn (+15.0%). Build: base
   5,483 + leasing 439 (+8%) + shophouse 383, the latter crediting ~30%
   of the guided VND1,575bn first-year gross profit (was ~22%). Now ~3%
   below MBS's 6,502.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QPsxWfyBSmSQjUzo5EDnm5
</commit_message>
<xml_diff>
--- a/Stock_Pick_and_Forecast_Aug26_MAS_RS_EN_updated.xlsx
+++ b/Stock_Pick_and_Forecast_Aug26_MAS_RS_EN_updated.xlsx
@@ -8,7 +8,6 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stock Pick" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Target Price and Forecast" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Assumptions" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191028" fullCalcOnLoad="1" iterate="1"/>
@@ -1163,7 +1162,7 @@
         <is>
           <t>FY25 NPAT hit a record VND6,446bn (+57.3% YoY), flattered by one-off financial income (chiefly the Vincom Center Nguyen Chi Thanh stake transfer); on an adjusted basis NPAT was VND4,694bn (+16.3% YoY). FY25 net revenue was VND8,712bn, with leasing revenue of VND8,400bn (+8.3% YoY). Momentum carried into 1Q26: net revenue VND2,574bn (+20.7% YoY) and NPAT VND1,606bn (+36.4% YoY).
 We forecast FY26F net revenue VND10,639bn (~5% above the VND10,132bn plan) but NPATMI of VND5,483bn only ~2% above the VND5,375bn target — i.e. +22.1% on FY25 revenue and +16.8% on adjusted FY25 NPAT (-13.9% against the one-off-inflated reported FY25 NPAT). The narrower profit beat reflects a net margin of 51.5% vs the ~53.0% implied by plan (~150bp dilution), as pre-operating costs and depreciation on newly opened GFA land ahead of full occupancy.
-FY27F NPATMI VND6,196bn (+13.0% YoY) rests on two identifiable drivers rather than trend growth, with the property leg deliberately haircut (see the Sources &amp; Assumptions tab for the build). (i) Mall lease-up: GFA opened late in 2026 — Vincom Plaza at Wonder City (~27,000 sqm, 3Q26) and J-Town My Lam (4Q26) — contributes only partially in FY26 and annualises in FY27, joined by Vincom Mega Mall Long An (Tay Ninh) due in 2027, against occupancy of 88.1% at end-2025 across 90 malls. (ii) Commercial property transfers: management guides this to become a new earnings driver from 2027, as the ~1,200 shophouses at Vinhomes Royal Island and Vinhomes Golden Avenue (VND5,480bn deposited for ~109,800 sqm; ~45% gross margin) are handed over — the segment is guided at only ~1.5-2% of FY26 revenue, so the step-up falls in FY27. We credit only ~22% of the ~VND1,575bn gross profit management guided for a full handover year, because the schedule has already slipped once (press guidance in Oct-2025 put the step-up in FY26; the Apr-2026 AGM moved it to FY27) and the model's own 'sale of investment properties' line has ranged from VND381bn to VND3,433bn historically. This leaves us ~5% below MBS (FY27 NPAT VND6,502bn, +19.2%), which assumes a fuller handover.</t>
+FY27F NPATMI VND6,305bn (+15.0% YoY) rests on two identifiable drivers rather than trend growth, with the property leg deliberately haircut. (i) Mall lease-up: GFA opened late in 2026 — Vincom Plaza at Wonder City (~27,000 sqm, 3Q26) and J-Town My Lam (4Q26) — contributes only partially in FY26 and annualises in FY27, joined by Vincom Mega Mall Long An (Tay Ninh) due in 2027, against occupancy of 88.1% at end-2025 across 90 malls. (ii) Commercial property transfers: management guides this to become a new earnings driver from 2027, as the ~1,200 shophouses at Vinhomes Royal Island and Vinhomes Golden Avenue (VND5,480bn deposited for ~109,800 sqm; ~45% gross margin) are handed over — the segment is guided at only ~1.5-2% of FY26 revenue, so the step-up falls in FY27. We credit only ~30% of the ~VND1,575bn gross profit management guided for a full handover year, because the schedule has already slipped once (press guidance in Oct-2025 put the step-up in FY26; the Apr-2026 AGM moved it to FY27) and the model's own 'sale of investment properties' line has ranged from VND381bn to VND3,433bn historically. This leaves us ~3% below MBS (FY27 NPAT VND6,502bn, +19.2%), which assumes a fuller handover.</t>
         </is>
       </c>
       <c r="D9" s="16" t="inlineStr">
@@ -1176,7 +1175,7 @@
       </c>
       <c r="E9" s="16" t="inlineStr">
         <is>
-          <t>- Commercial property transfers are a potential new earnings stream from 2027: ~1,200 shophouses at Vinhomes Royal Island and Golden Avenue (VND5,480bn deposited, ~45% gross margin) under the Vincom Collection format. We treat this as optionality, not a base-case engine - our forecast credits only ~22% of the guided first-year gross profit.
+          <t>- Commercial property transfers are a potential new earnings stream from 2027: ~1,200 shophouses at Vinhomes Royal Island and Golden Avenue (VND5,480bn deposited, ~45% gross margin) under the Vincom Collection format. We treat this as optionality, not a base-case engine - our forecast credits only ~30% of the guided first-year gross profit.
 - Mall pipeline: Wonder City (~27,000 sqm) and J-Town My Lam open in 2H26 and annualise in 2027; Vincom Mega Mall Long An follows in 2027, with management flagging 2028 as the breakout year as transport-infrastructure-linked projects complete (GFA target ~3.5mn sqm post-2030 vs ~1.9mn now).
 - Occupancy maximization across 90 operating malls (88.1% at end-2025) supports leasing revenue growth.
 - First cash dividend in 7 years (10% of par, ~VND2.2tn, paid Jul 2026) signals a shareholder-return shift.
@@ -1187,19 +1186,19 @@
         <v>5483</v>
       </c>
       <c r="G9" s="61" t="n">
-        <v>6196</v>
+        <v>6305</v>
       </c>
       <c r="H9" s="62" t="n">
         <v>-0.1388706531264823</v>
       </c>
       <c r="I9" s="62" t="n">
-        <v>0.13003830020062</v>
+        <v>0.1499179281415284</v>
       </c>
       <c r="J9" s="63" t="n">
         <v>11.89256159037024</v>
       </c>
       <c r="K9" s="63" t="n">
-        <v>10.52403408650743</v>
+        <v>10.34209598731166</v>
       </c>
       <c r="L9" s="63" t="n">
         <v>1.228188684873102</v>
@@ -1709,7 +1708,7 @@
         <v>5483</v>
       </c>
       <c r="E18" s="15" t="n">
-        <v>6196</v>
+        <v>6305</v>
       </c>
     </row>
     <row r="19" ht="15.6" customFormat="1" customHeight="1" s="1">
@@ -2232,1144 +2231,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G38"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="52" customWidth="1" min="6" max="6"/>
-    <col width="62" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="68" t="inlineStr">
-        <is>
-          <t>SOURCES &amp; ASSUMPTIONS — provenance record for every figure used in the Stock Pick tab</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="28" customHeight="1">
-      <c r="A2" s="69" t="inlineStr">
-        <is>
-          <t>RULE: no figure enters a client-facing cell without a source tag below. MODEL = a cell in our own model · COMPANY = company disclosure/plan/AGM · PRESS = media report (outlet + date) · MAS = our estimate, which must show its build · UNVERIFIED = single unconfirmed source, flagged in red.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="70" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B4" s="70" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="C4" s="70" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-      <c r="D4" s="70" t="inlineStr">
-        <is>
-          <t>Unit</t>
-        </is>
-      </c>
-      <c r="E4" s="70" t="inlineStr">
-        <is>
-          <t>Source type</t>
-        </is>
-      </c>
-      <c r="F4" s="70" t="inlineStr">
-        <is>
-          <t>Source detail / date</t>
-        </is>
-      </c>
-      <c r="G4" s="70" t="inlineStr">
-        <is>
-          <t>Status &amp; notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="71" t="inlineStr"/>
-      <c r="B5" s="72" t="inlineStr">
-        <is>
-          <t>VRE — FY25 REPORTED</t>
-        </is>
-      </c>
-      <c r="C5" s="71" t="inlineStr"/>
-      <c r="D5" s="71" t="inlineStr"/>
-      <c r="E5" s="71" t="inlineStr"/>
-      <c r="F5" s="71" t="inlineStr"/>
-      <c r="G5" s="71" t="inlineStr"/>
-    </row>
-    <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="73" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B6" s="73" t="inlineStr">
-        <is>
-          <t>Net revenue FY25</t>
-        </is>
-      </c>
-      <c r="C6" s="73" t="inlineStr">
-        <is>
-          <t>8,712</t>
-        </is>
-      </c>
-      <c r="D6" s="73" t="inlineStr">
-        <is>
-          <t>VNDbn</t>
-        </is>
-      </c>
-      <c r="E6" s="73" t="inlineStr">
-        <is>
-          <t>PRESS + COMPANY</t>
-        </is>
-      </c>
-      <c r="F6" s="74" t="inlineStr">
-        <is>
-          <t>Media reports of FY25 results; cross-checks to the FY26 plan (VND10,132bn stated as +16% YoY -&gt; implies 8,734)</t>
-        </is>
-      </c>
-      <c r="G6" s="74" t="inlineStr">
-        <is>
-          <t>RECONCILED. NOT an adjusted figure — the FY25 one-offs sat in financial income, below the revenue line. Model Summary!K157 shows 9,074 but that column is a 2025F forecast, not actual.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="73" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B7" s="73" t="inlineStr">
-        <is>
-          <t>Leasing revenue FY25</t>
-        </is>
-      </c>
-      <c r="C7" s="73" t="inlineStr">
-        <is>
-          <t>8,400</t>
-        </is>
-      </c>
-      <c r="D7" s="73" t="inlineStr">
-        <is>
-          <t>VNDbn</t>
-        </is>
-      </c>
-      <c r="E7" s="73" t="inlineStr">
-        <is>
-          <t>PRESS</t>
-        </is>
-      </c>
-      <c r="F7" s="74" t="inlineStr">
-        <is>
-          <t>FY25 results coverage, +8.3% YoY</t>
-        </is>
-      </c>
-      <c r="G7" s="74" t="inlineStr">
-        <is>
-          <t>Single source; consistent with model leasing 2025F of 8,311.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="73" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B8" s="73" t="inlineStr">
-        <is>
-          <t>NPAT FY25 (reported)</t>
-        </is>
-      </c>
-      <c r="C8" s="73" t="inlineStr">
-        <is>
-          <t>6,446</t>
-        </is>
-      </c>
-      <c r="D8" s="73" t="inlineStr">
-        <is>
-          <t>VNDbn</t>
-        </is>
-      </c>
-      <c r="E8" s="73" t="inlineStr">
-        <is>
-          <t>COMPANY</t>
-        </is>
-      </c>
-      <c r="F8" s="74" t="inlineStr">
-        <is>
-          <t>FY25 results announcement, +57.3% YoY</t>
-        </is>
-      </c>
-      <c r="G8" s="74" t="inlineStr">
-        <is>
-          <t>Confirmed by multiple outlets.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="73" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B9" s="73" t="inlineStr">
-        <is>
-          <t>NPAT FY25 (adjusted)</t>
-        </is>
-      </c>
-      <c r="C9" s="73" t="inlineStr">
-        <is>
-          <t>4,694</t>
-        </is>
-      </c>
-      <c r="D9" s="73" t="inlineStr">
-        <is>
-          <t>VNDbn</t>
-        </is>
-      </c>
-      <c r="E9" s="73" t="inlineStr">
-        <is>
-          <t>COMPANY</t>
-        </is>
-      </c>
-      <c r="F9" s="74" t="inlineStr">
-        <is>
-          <t>Ex one-off financial income (Vincom Center Nguyen Chi Thanh stake transfer), +16.3% YoY</t>
-        </is>
-      </c>
-      <c r="G9" s="74" t="inlineStr">
-        <is>
-          <t>"Adjusted" applies to PROFIT ONLY.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="73" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B10" s="73" t="inlineStr">
-        <is>
-          <t>NPAT FY25 (our model base)</t>
-        </is>
-      </c>
-      <c r="C10" s="73" t="inlineStr">
-        <is>
-          <t>6,367</t>
-        </is>
-      </c>
-      <c r="D10" s="73" t="inlineStr">
-        <is>
-          <t>VNDbn</t>
-        </is>
-      </c>
-      <c r="E10" s="73" t="inlineStr">
-        <is>
-          <t>MODEL</t>
-        </is>
-      </c>
-      <c r="F10" s="74" t="inlineStr">
-        <is>
-          <t>VRE_1Q26_v2_linked2.xlsx Summary!K158</t>
-        </is>
-      </c>
-      <c r="G10" s="74" t="inlineStr">
-        <is>
-          <t>Used as the col-H growth denominator for cross-ticker consistency; differs from the 6,446 reported.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="71" t="inlineStr"/>
-      <c r="B11" s="72" t="inlineStr">
-        <is>
-          <t>VRE — 1Q26 REPORTED</t>
-        </is>
-      </c>
-      <c r="C11" s="71" t="inlineStr"/>
-      <c r="D11" s="71" t="inlineStr"/>
-      <c r="E11" s="71" t="inlineStr"/>
-      <c r="F11" s="71" t="inlineStr"/>
-      <c r="G11" s="71" t="inlineStr"/>
-    </row>
-    <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="73" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="B12" s="73" t="inlineStr">
-        <is>
-          <t>Net revenue 1Q26</t>
-        </is>
-      </c>
-      <c r="C12" s="73" t="inlineStr">
-        <is>
-          <t>2,574</t>
-        </is>
-      </c>
-      <c r="D12" s="73" t="inlineStr">
-        <is>
-          <t>VNDbn</t>
-        </is>
-      </c>
-      <c r="E12" s="73" t="inlineStr">
-        <is>
-          <t>PRESS</t>
-        </is>
-      </c>
-      <c r="F12" s="74" t="inlineStr">
-        <is>
-          <t>1Q26 results coverage, +20.7% YoY</t>
-        </is>
-      </c>
-      <c r="G12" s="74" t="inlineStr">
-        <is>
-          <t>Reported figure. Earlier draft wrongly labelled this "adjusted" — corrected.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="73" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="B13" s="73" t="inlineStr">
-        <is>
-          <t>NPAT 1Q26</t>
-        </is>
-      </c>
-      <c r="C13" s="73" t="inlineStr">
-        <is>
-          <t>1,606</t>
-        </is>
-      </c>
-      <c r="D13" s="73" t="inlineStr">
-        <is>
-          <t>VNDbn</t>
-        </is>
-      </c>
-      <c r="E13" s="73" t="inlineStr">
-        <is>
-          <t>PRESS</t>
-        </is>
-      </c>
-      <c r="F13" s="74" t="inlineStr">
-        <is>
-          <t>1Q26 results coverage, +36.4% YoY</t>
-        </is>
-      </c>
-      <c r="G13" s="74" t="inlineStr">
-        <is>
-          <t>Confirmed by multiple outlets.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="71" t="inlineStr"/>
-      <c r="B14" s="72" t="inlineStr">
-        <is>
-          <t>VRE — FY26F</t>
-        </is>
-      </c>
-      <c r="C14" s="71" t="inlineStr"/>
-      <c r="D14" s="71" t="inlineStr"/>
-      <c r="E14" s="71" t="inlineStr"/>
-      <c r="F14" s="71" t="inlineStr"/>
-      <c r="G14" s="71" t="inlineStr"/>
-    </row>
-    <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="73" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="B15" s="73" t="inlineStr">
-        <is>
-          <t>FY26 revenue plan</t>
-        </is>
-      </c>
-      <c r="C15" s="73" t="inlineStr">
-        <is>
-          <t>10,132</t>
-        </is>
-      </c>
-      <c r="D15" s="73" t="inlineStr">
-        <is>
-          <t>VNDbn</t>
-        </is>
-      </c>
-      <c r="E15" s="73" t="inlineStr">
-        <is>
-          <t>COMPANY</t>
-        </is>
-      </c>
-      <c r="F15" s="74" t="inlineStr">
-        <is>
-          <t>2026 AGM, 23-Apr-2026</t>
-        </is>
-      </c>
-      <c r="G15" s="74" t="inlineStr">
-        <is>
-          <t>Board-approved plan.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="73" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="B16" s="73" t="inlineStr">
-        <is>
-          <t>FY26 NPAT plan</t>
-        </is>
-      </c>
-      <c r="C16" s="73" t="inlineStr">
-        <is>
-          <t>5,375</t>
-        </is>
-      </c>
-      <c r="D16" s="73" t="inlineStr">
-        <is>
-          <t>VNDbn</t>
-        </is>
-      </c>
-      <c r="E16" s="73" t="inlineStr">
-        <is>
-          <t>COMPANY</t>
-        </is>
-      </c>
-      <c r="F16" s="74" t="inlineStr">
-        <is>
-          <t>2026 AGM, 23-Apr-2026</t>
-        </is>
-      </c>
-      <c r="G16" s="74" t="inlineStr">
-        <is>
-          <t>Board-approved plan.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="73" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="B17" s="73" t="inlineStr">
-        <is>
-          <t>MAS FY26F net revenue</t>
-        </is>
-      </c>
-      <c r="C17" s="73" t="inlineStr">
-        <is>
-          <t>10,639</t>
-        </is>
-      </c>
-      <c r="D17" s="73" t="inlineStr">
-        <is>
-          <t>VNDbn</t>
-        </is>
-      </c>
-      <c r="E17" s="73" t="inlineStr">
-        <is>
-          <t>MAS</t>
-        </is>
-      </c>
-      <c r="F17" s="74">
-        <f> plan x 1.05, per analyst instruction</f>
-        <v/>
-      </c>
-      <c r="G17" s="74" t="inlineStr">
-        <is>
-          <t>Build: 10,132 x 1.05.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="73" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="B18" s="73" t="inlineStr">
-        <is>
-          <t>MAS FY26F NPATMI</t>
-        </is>
-      </c>
-      <c r="C18" s="73" t="inlineStr">
-        <is>
-          <t>5,483</t>
-        </is>
-      </c>
-      <c r="D18" s="73" t="inlineStr">
-        <is>
-          <t>VNDbn</t>
-        </is>
-      </c>
-      <c r="E18" s="73" t="inlineStr">
-        <is>
-          <t>MAS</t>
-        </is>
-      </c>
-      <c r="F18" s="74">
-        <f> plan x 1.02, per analyst instruction</f>
-        <v/>
-      </c>
-      <c r="G18" s="74" t="inlineStr">
-        <is>
-          <t>Build: 5,375 x 1.02. Implies a 51.5% net margin vs ~53.0% in plan.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="71" t="inlineStr"/>
-      <c r="B19" s="72" t="inlineStr">
-        <is>
-          <t>VRE — FY27F BUILD (adopted)</t>
-        </is>
-      </c>
-      <c r="C19" s="71" t="inlineStr"/>
-      <c r="D19" s="71" t="inlineStr"/>
-      <c r="E19" s="71" t="inlineStr"/>
-      <c r="F19" s="71" t="inlineStr"/>
-      <c r="G19" s="71" t="inlineStr"/>
-    </row>
-    <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="73" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="B20" s="73" t="inlineStr">
-        <is>
-          <t>FY26F NPATMI base</t>
-        </is>
-      </c>
-      <c r="C20" s="73" t="inlineStr">
-        <is>
-          <t>5,483</t>
-        </is>
-      </c>
-      <c r="D20" s="73" t="inlineStr">
-        <is>
-          <t>VNDbn</t>
-        </is>
-      </c>
-      <c r="E20" s="73" t="inlineStr">
-        <is>
-          <t>MAS</t>
-        </is>
-      </c>
-      <c r="F20" s="74" t="inlineStr">
-        <is>
-          <t>row 11</t>
-        </is>
-      </c>
-      <c r="G20" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="30" customHeight="1">
-      <c r="A21" s="73" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="B21" s="73" t="inlineStr">
-        <is>
-          <t>+ organic leasing growth</t>
-        </is>
-      </c>
-      <c r="C21" s="73" t="inlineStr">
-        <is>
-          <t>439</t>
-        </is>
-      </c>
-      <c r="D21" s="73" t="inlineStr">
-        <is>
-          <t>VNDbn</t>
-        </is>
-      </c>
-      <c r="E21" s="73" t="inlineStr">
-        <is>
-          <t>MAS</t>
-        </is>
-      </c>
-      <c r="F21" s="74" t="inlineStr">
-        <is>
-          <t>+8.0% on base: 2026 GFA additions annualise; occupancy 88.1% (end-2025) recovering</t>
-        </is>
-      </c>
-      <c r="G21" s="74" t="inlineStr">
-        <is>
-          <t>GFA +5.2% in the model; +8% profit growth assumes modest operating leverage.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="75" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="B22" s="75" t="inlineStr">
-        <is>
-          <t>+ shophouse handover</t>
-        </is>
-      </c>
-      <c r="C22" s="75" t="inlineStr">
-        <is>
-          <t>274</t>
-        </is>
-      </c>
-      <c r="D22" s="75" t="inlineStr">
-        <is>
-          <t>VNDbn</t>
-        </is>
-      </c>
-      <c r="E22" s="75" t="inlineStr">
-        <is>
-          <t>MAS</t>
-        </is>
-      </c>
-      <c r="F22" s="76" t="inlineStr">
-        <is>
-          <t>~22% of the VND1,575bn guided first-year gross profit, taxed at 20%</t>
-        </is>
-      </c>
-      <c r="G22" s="76" t="inlineStr">
-        <is>
-          <t>DELIBERATELY HAIRCUT — see conflicts below.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="30" customHeight="1">
-      <c r="A23" s="77" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="B23" s="77">
-        <f> FY27F NPATMI</f>
-        <v/>
-      </c>
-      <c r="C23" s="77" t="inlineStr">
-        <is>
-          <t>6,196</t>
-        </is>
-      </c>
-      <c r="D23" s="77" t="inlineStr">
-        <is>
-          <t>VNDbn</t>
-        </is>
-      </c>
-      <c r="E23" s="77" t="inlineStr">
-        <is>
-          <t>MAS</t>
-        </is>
-      </c>
-      <c r="F23" s="78" t="inlineStr">
-        <is>
-          <t>rows 12+13+14</t>
-        </is>
-      </c>
-      <c r="G23" s="78" t="inlineStr">
-        <is>
-          <t>+13.0% YoY.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="71" t="inlineStr"/>
-      <c r="B24" s="72" t="inlineStr">
-        <is>
-          <t>FY27F SCENARIOS</t>
-        </is>
-      </c>
-      <c r="C24" s="71" t="inlineStr"/>
-      <c r="D24" s="71" t="inlineStr"/>
-      <c r="E24" s="71" t="inlineStr"/>
-      <c r="F24" s="71" t="inlineStr"/>
-      <c r="G24" s="71" t="inlineStr"/>
-    </row>
-    <row r="25" ht="30" customHeight="1">
-      <c r="A25" s="73" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="B25" s="73" t="inlineStr">
-        <is>
-          <t>Low — leasing only, no shophouse</t>
-        </is>
-      </c>
-      <c r="C25" s="73" t="inlineStr">
-        <is>
-          <t>5,922</t>
-        </is>
-      </c>
-      <c r="D25" s="73" t="inlineStr">
-        <is>
-          <t>VNDbn</t>
-        </is>
-      </c>
-      <c r="E25" s="73" t="inlineStr">
-        <is>
-          <t>MAS</t>
-        </is>
-      </c>
-      <c r="F25" s="74" t="inlineStr">
-        <is>
-          <t>5,483 x 1.08</t>
-        </is>
-      </c>
-      <c r="G25" s="74" t="inlineStr">
-        <is>
-          <t>+8.0% YoY.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="30" customHeight="1">
-      <c r="A26" s="77" t="inlineStr">
-        <is>
-          <t>17</t>
-        </is>
-      </c>
-      <c r="B26" s="77" t="inlineStr">
-        <is>
-          <t>Base — adopted</t>
-        </is>
-      </c>
-      <c r="C26" s="77" t="inlineStr">
-        <is>
-          <t>6,196</t>
-        </is>
-      </c>
-      <c r="D26" s="77" t="inlineStr">
-        <is>
-          <t>VNDbn</t>
-        </is>
-      </c>
-      <c r="E26" s="77" t="inlineStr">
-        <is>
-          <t>MAS</t>
-        </is>
-      </c>
-      <c r="F26" s="78" t="inlineStr">
-        <is>
-          <t>row 15</t>
-        </is>
-      </c>
-      <c r="G26" s="78" t="inlineStr">
-        <is>
-          <t>+13.0% YoY.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="30" customHeight="1">
-      <c r="A27" s="73" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
-      </c>
-      <c r="B27" s="73" t="inlineStr">
-        <is>
-          <t>High — full handover</t>
-        </is>
-      </c>
-      <c r="C27" s="73" t="inlineStr">
-        <is>
-          <t>6,580</t>
-        </is>
-      </c>
-      <c r="D27" s="73" t="inlineStr">
-        <is>
-          <t>VNDbn</t>
-        </is>
-      </c>
-      <c r="E27" s="73" t="inlineStr">
-        <is>
-          <t>MAS</t>
-        </is>
-      </c>
-      <c r="F27" s="74" t="inlineStr">
-        <is>
-          <t>5,483 x 1.20</t>
-        </is>
-      </c>
-      <c r="G27" s="74" t="inlineStr">
-        <is>
-          <t>+20.0% YoY. MBS forecasts 6,502 (+19.2%) on a similar full-handover view.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="71" t="inlineStr"/>
-      <c r="B28" s="72" t="inlineStr">
-        <is>
-          <t>SHOPHOUSE PIPELINE — underlying facts</t>
-        </is>
-      </c>
-      <c r="C28" s="71" t="inlineStr"/>
-      <c r="D28" s="71" t="inlineStr"/>
-      <c r="E28" s="71" t="inlineStr"/>
-      <c r="F28" s="71" t="inlineStr"/>
-      <c r="G28" s="71" t="inlineStr"/>
-    </row>
-    <row r="29" ht="30" customHeight="1">
-      <c r="A29" s="73" t="inlineStr">
-        <is>
-          <t>19</t>
-        </is>
-      </c>
-      <c r="B29" s="73" t="inlineStr">
-        <is>
-          <t>Deposit paid for shophouse land</t>
-        </is>
-      </c>
-      <c r="C29" s="73" t="inlineStr">
-        <is>
-          <t>5,480</t>
-        </is>
-      </c>
-      <c r="D29" s="73" t="inlineStr">
-        <is>
-          <t>VNDbn</t>
-        </is>
-      </c>
-      <c r="E29" s="73" t="inlineStr">
-        <is>
-          <t>PRESS</t>
-        </is>
-      </c>
-      <c r="F29" s="74" t="inlineStr">
-        <is>
-          <t>MarketTimes; deposit made end-2024 for ~109,800 sqm net floor</t>
-        </is>
-      </c>
-      <c r="G29" s="74" t="inlineStr">
-        <is>
-          <t>~1,200 units at Vinhomes Royal Island (~1,000) + Golden Avenue (~280).</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="30" customHeight="1">
-      <c r="A30" s="73" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="B30" s="73" t="inlineStr">
-        <is>
-          <t>Guided gross margin</t>
-        </is>
-      </c>
-      <c r="C30" s="73" t="inlineStr">
-        <is>
-          <t>45</t>
-        </is>
-      </c>
-      <c r="D30" s="73" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="E30" s="73" t="inlineStr">
-        <is>
-          <t>PRESS</t>
-        </is>
-      </c>
-      <c r="F30" s="74" t="inlineStr">
-        <is>
-          <t>Broker/press coverage of the shophouse programme</t>
-        </is>
-      </c>
-      <c r="G30" s="74" t="inlineStr">
-        <is>
-          <t>Single-source estimate.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="30" customHeight="1">
-      <c r="A31" s="73" t="inlineStr">
-        <is>
-          <t>21</t>
-        </is>
-      </c>
-      <c r="B31" s="73" t="inlineStr">
-        <is>
-          <t>Guided gross profit, first handover yr</t>
-        </is>
-      </c>
-      <c r="C31" s="73" t="inlineStr">
-        <is>
-          <t>1,575</t>
-        </is>
-      </c>
-      <c r="D31" s="73" t="inlineStr">
-        <is>
-          <t>VNDbn</t>
-        </is>
-      </c>
-      <c r="E31" s="73" t="inlineStr">
-        <is>
-          <t>PRESS</t>
-        </is>
-      </c>
-      <c r="F31" s="74" t="inlineStr">
-        <is>
-          <t>CafeF, 10-Oct-2025</t>
-        </is>
-      </c>
-      <c r="G31" s="79" t="inlineStr">
-        <is>
-          <t>UNVERIFIED against company disclosure — treat as indicative.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="30" customHeight="1">
-      <c r="A32" s="73" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="B32" s="73" t="inlineStr">
-        <is>
-          <t>Vincom Collection share of FY26 rev</t>
-        </is>
-      </c>
-      <c r="C32" s="73" t="inlineStr">
-        <is>
-          <t>1.5-2</t>
-        </is>
-      </c>
-      <c r="D32" s="73" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="E32" s="73" t="inlineStr">
-        <is>
-          <t>COMPANY</t>
-        </is>
-      </c>
-      <c r="F32" s="74" t="inlineStr">
-        <is>
-          <t>2026 AGM, 23-Apr-2026</t>
-        </is>
-      </c>
-      <c r="G32" s="74" t="inlineStr">
-        <is>
-          <t>Confirms the FY26 property contribution is small.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="71" t="inlineStr"/>
-      <c r="B33" s="72" t="inlineStr">
-        <is>
-          <t>KNOWN CONFLICTS &amp; OPEN ITEMS</t>
-        </is>
-      </c>
-      <c r="C33" s="71" t="inlineStr"/>
-      <c r="D33" s="71" t="inlineStr"/>
-      <c r="E33" s="71" t="inlineStr"/>
-      <c r="F33" s="71" t="inlineStr"/>
-      <c r="G33" s="71" t="inlineStr"/>
-    </row>
-    <row r="34" ht="30" customHeight="1">
-      <c r="A34" s="73" t="inlineStr">
-        <is>
-          <t>C1</t>
-        </is>
-      </c>
-      <c r="B34" s="73" t="inlineStr">
-        <is>
-          <t>Shophouse timing has already slipped</t>
-        </is>
-      </c>
-      <c r="C34" s="73" t="inlineStr"/>
-      <c r="D34" s="73" t="inlineStr"/>
-      <c r="E34" s="73" t="inlineStr"/>
-      <c r="F34" s="74" t="inlineStr">
-        <is>
-          <t>CafeF (Oct-2025) put the profit step-up in FY26; the Apr-2026 AGM moved it to "from 2027"</t>
-        </is>
-      </c>
-      <c r="G34" s="79" t="inlineStr">
-        <is>
-          <t>Reason for the haircut in row 14.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="30" customHeight="1">
-      <c r="A35" s="73" t="inlineStr">
-        <is>
-          <t>C2</t>
-        </is>
-      </c>
-      <c r="B35" s="73" t="inlineStr">
-        <is>
-          <t>Historic volatility of the property line</t>
-        </is>
-      </c>
-      <c r="C35" s="73" t="inlineStr">
-        <is>
-          <t>381-3,433</t>
-        </is>
-      </c>
-      <c r="D35" s="73" t="inlineStr">
-        <is>
-          <t>VNDbn</t>
-        </is>
-      </c>
-      <c r="E35" s="73" t="inlineStr">
-        <is>
-          <t>MODEL</t>
-        </is>
-      </c>
-      <c r="F35" s="74" t="inlineStr">
-        <is>
-          <t>VRE model IS!r78 "Sale of investment properties", FY18-FY24 range</t>
-        </is>
-      </c>
-      <c r="G35" s="79" t="inlineStr">
-        <is>
-          <t>Handover timing is the single largest swing factor in FY27.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="30" customHeight="1">
-      <c r="A36" s="73" t="inlineStr">
-        <is>
-          <t>C3</t>
-        </is>
-      </c>
-      <c r="B36" s="73" t="inlineStr">
-        <is>
-          <t>BVPS / P-B basis</t>
-        </is>
-      </c>
-      <c r="C36" s="73" t="inlineStr">
-        <is>
-          <t>22,798 / 25,513</t>
-        </is>
-      </c>
-      <c r="D36" s="73" t="inlineStr">
-        <is>
-          <t>VND</t>
-        </is>
-      </c>
-      <c r="E36" s="73" t="inlineStr">
-        <is>
-          <t>MODEL</t>
-        </is>
-      </c>
-      <c r="F36" s="74" t="inlineStr">
-        <is>
-          <t>VRE model BS!L136 / M136</t>
-        </is>
-      </c>
-      <c r="G36" s="79" t="inlineStr">
-        <is>
-          <t>Model balance sheet embeds LOWER earnings than the forecasts overridden into the Stock Pick tab, so P/B is modestly overstated.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="30" customHeight="1">
-      <c r="A37" s="73" t="inlineStr">
-        <is>
-          <t>C4</t>
-        </is>
-      </c>
-      <c r="B37" s="73" t="inlineStr">
-        <is>
-          <t>FY28F</t>
-        </is>
-      </c>
-      <c r="C37" s="73" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="D37" s="73" t="inlineStr"/>
-      <c r="E37" s="73" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F37" s="74" t="inlineStr">
-        <is>
-          <t>VRE model and Stock Pick tab both stop at FY27F</t>
-        </is>
-      </c>
-      <c r="G37" s="74" t="inlineStr">
-        <is>
-          <t>No FY28 figure exists; none has been estimated.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="30" customHeight="1">
-      <c r="A38" s="73" t="inlineStr">
-        <is>
-          <t>C5</t>
-        </is>
-      </c>
-      <c r="B38" s="73" t="inlineStr">
-        <is>
-          <t>A property-led FY27 creates a high FY28 base</t>
-        </is>
-      </c>
-      <c r="C38" s="73" t="inlineStr"/>
-      <c r="D38" s="73" t="inlineStr"/>
-      <c r="E38" s="73" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F38" s="74" t="inlineStr">
-        <is>
-          <t>Analytical note</t>
-        </is>
-      </c>
-      <c r="G38" s="74" t="inlineStr">
-        <is>
-          <t>Same distortion FY25 one-offs created for FY26 optics.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A2:G2"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Condense VRE growth narrative by ~35%
Tightened the Growth cell from 2,043 to 1,324 characters by cutting
connective phrasing, not substance. All figures retained except the
~109,800 sqm net floor area (redundant beside the ~1,200 unit count);
the VND381-3,433bn property-line range is now expressed as a range.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QPsxWfyBSmSQjUzo5EDnm5
</commit_message>
<xml_diff>
--- a/Stock_Pick_and_Forecast_Aug26_MAS_RS_EN_updated.xlsx
+++ b/Stock_Pick_and_Forecast_Aug26_MAS_RS_EN_updated.xlsx
@@ -1160,9 +1160,9 @@
       </c>
       <c r="C9" s="17" t="inlineStr">
         <is>
-          <t>FY25 NPAT hit a record VND6,446bn (+57.3% YoY), flattered by one-off financial income (chiefly the Vincom Center Nguyen Chi Thanh stake transfer); on an adjusted basis NPAT was VND4,694bn (+16.3% YoY). FY25 net revenue was VND8,712bn, with leasing revenue of VND8,400bn (+8.3% YoY). Momentum carried into 1Q26: net revenue VND2,574bn (+20.7% YoY) and NPAT VND1,606bn (+36.4% YoY).
-We forecast FY26F net revenue VND10,639bn (~5% above the VND10,132bn plan) but NPATMI of VND5,483bn only ~2% above the VND5,375bn target — i.e. +22.1% on FY25 revenue and +16.8% on adjusted FY25 NPAT (-13.9% against the one-off-inflated reported FY25 NPAT). The narrower profit beat reflects a net margin of 51.5% vs the ~53.0% implied by plan (~150bp dilution), as pre-operating costs and depreciation on newly opened GFA land ahead of full occupancy.
-FY27F NPATMI VND6,305bn (+15.0% YoY) rests on two identifiable drivers rather than trend growth, with the property leg deliberately haircut. (i) Mall lease-up: GFA opened late in 2026 — Vincom Plaza at Wonder City (~27,000 sqm, 3Q26) and J-Town My Lam (4Q26) — contributes only partially in FY26 and annualises in FY27, joined by Vincom Mega Mall Long An (Tay Ninh) due in 2027, against occupancy of 88.1% at end-2025 across 90 malls. (ii) Commercial property transfers: management guides this to become a new earnings driver from 2027, as the ~1,200 shophouses at Vinhomes Royal Island and Vinhomes Golden Avenue (VND5,480bn deposited for ~109,800 sqm; ~45% gross margin) are handed over — the segment is guided at only ~1.5-2% of FY26 revenue, so the step-up falls in FY27. We credit only ~30% of the ~VND1,575bn gross profit management guided for a full handover year, because the schedule has already slipped once (press guidance in Oct-2025 put the step-up in FY26; the Apr-2026 AGM moved it to FY27) and the model's own 'sale of investment properties' line has ranged from VND381bn to VND3,433bn historically. This leaves us ~3% below MBS (FY27 NPAT VND6,502bn, +19.2%), which assumes a fuller handover.</t>
+          <t>FY25 NPAT was a record VND6,446bn (+57.3%), flattered by one-off financial income (Vincom Center Nguyen Chi Thanh stake transfer); adjusted NPAT VND4,694bn (+16.3%). FY25 net revenue VND8,712bn, leasing VND8,400bn (+8.3%). 1Q26 carried the momentum: revenue VND2,574bn (+20.7%), NPAT VND1,606bn (+36.4%).
+FY26F net revenue VND10,639bn (~5% above the VND10,132bn plan) but NPATMI VND5,483bn only ~2% above the VND5,375bn target — +22.1% on FY25 revenue and +16.8% on adjusted FY25 NPAT (-13.9% vs the one-off-inflated reported base). The narrower profit beat is ~150bp of margin dilution (51.5% vs ~53.0% planned), from pre-operating costs and depreciation on newly opened GFA.
+FY27F NPATMI VND6,305bn (+15.0%) rests on two drivers, with the property leg haircut. (i) Lease-up: Wonder City (~27,000 sqm, 3Q26) and J-Town My Lam (4Q26) annualise, plus Vincom Mega Mall Long An in 2027; occupancy 88.1% across 90 malls. (ii) Property transfers: ~1,200 shophouses at Vinhomes Royal Island and Golden Avenue (VND5,480bn deposited, ~45% GM), guided as a new driver from 2027 (only ~1.5-2% of FY26 revenue). We credit ~30% of the guided VND1,575bn first-year gross profit — the schedule already slipped from FY26 to FY27, and the property line has ranged VND381-3,433bn historically — leaving us ~3% below MBS (VND6,502bn, +19.2%).</t>
         </is>
       </c>
       <c r="D9" s="16" t="inlineStr">

</xml_diff>